<commit_message>
Publish Intermediate M04 after technical validation
</commit_message>
<xml_diff>
--- a/downloads/exercises/intermedio-m04-m04-l03-practice-01.xlsx
+++ b/downloads/exercises/intermedio-m04-m04-l03-practice-01.xlsx
@@ -349,7 +349,7 @@
         <x:v>Días calendario incl.</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>No laborables</x:v>
+        <x:v>No laborables (con signo)</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
         <x:v>Caso</x:v>
@@ -518,12 +518,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>2. Calcula días calendario incluyendo ambas fechas con DIAS + 1.</x:v>
+        <x:v>2. Incluye ambas fechas: si la fecha final es igual o posterior a la inicial, usa DIAS(final;inicial) + 1; si es anterior, usa DIAS(final;inicial) - 1. El signo indica el orden del intervalo.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="str">
-        <x:v>3. Compara para identificar cuántos días no laborables quedaron fuera.</x:v>
+        <x:v>3. Resta días calendario incluidos menos días laborables: la diferencia conserva el signo del intervalo. En sentido inverso también es negativa; su magnitud es la cantidad física de días no laborables.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>